<commit_message>
SPM-52: bug test case added
</commit_message>
<xml_diff>
--- a/docs/test-cases/SPM-52_Test_Cases.xlsx
+++ b/docs/test-cases/SPM-52_Test_Cases.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="600" firstSheet="1" activeTab="10" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
@@ -17,7 +17,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC08" sheetId="9" state="visible" r:id="rId9"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC09" sheetId="10" state="visible" r:id="rId10"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC10" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TC11" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Bug Test Cases" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -26,10 +26,8 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
-    <numFmt numFmtId="164" formatCode="yyyy-mm-dd"/>
-    <numFmt numFmtId="165" formatCode="yyyy-mm-dd h:mm:ss"/>
-    <numFmt numFmtId="166" formatCode="yyyy\-mm\-dd"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
   <fonts count="6">
     <font>
@@ -40,6 +38,7 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
       <color theme="1"/>
       <sz val="10"/>
@@ -47,21 +46,25 @@
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <color theme="1"/>
       <sz val="10"/>
       <scheme val="minor"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <b val="1"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <sz val="10"/>
     </font>
     <font>
       <name val="Arial"/>
+      <family val="2"/>
       <color rgb="FF1155CC"/>
       <sz val="10"/>
       <u val="single"/>
@@ -116,44 +119,69 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
     <border>
       <left/>
       <right/>
-      <top style="thin"/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
       <diagonal/>
     </border>
     <border>
       <left/>
-      <right style="thin"/>
-      <top style="thin"/>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
       <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
       <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -164,8 +192,6 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
@@ -181,7 +207,14 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="166" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -460,8 +493,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F24"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:F23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="12.5"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="20" customWidth="1" min="2" max="2"/>
@@ -472,544 +505,510 @@
   </cols>
   <sheetData>
     <row r="1" ht="31" customHeight="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="16" t="inlineStr">
         <is>
           <t>Story</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="16" t="inlineStr">
         <is>
           <t>SPM-52: As an Attendee, I want to withdraw from an event I registered for so that my place can become available again where permitted</t>
         </is>
       </c>
-      <c r="C1" s="8" t="n"/>
-      <c r="D1" s="8" t="n"/>
-      <c r="E1" s="8" t="n"/>
-      <c r="F1" s="9" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" s="7" t="inlineStr">
+      <c r="C1" s="14" t="n"/>
+      <c r="D1" s="14" t="n"/>
+      <c r="E1" s="14" t="n"/>
+      <c r="F1" s="15" t="n"/>
+    </row>
+    <row r="3" ht="13" customHeight="1">
+      <c r="A3" s="16" t="inlineStr">
         <is>
           <t>Sheet</t>
         </is>
       </c>
-      <c r="B3" s="7" t="inlineStr">
+      <c r="B3" s="16" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" s="16" t="inlineStr">
         <is>
           <t>Title</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
         <is>
           <t>Linked AC</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="E3" s="16" t="inlineStr">
         <is>
           <t>Type</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="F3" s="16" t="inlineStr">
         <is>
           <t>Source</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="10" t="inlineStr">
+    <row r="4" ht="25" customHeight="1">
+      <c r="A4" s="8" t="inlineStr">
         <is>
           <t>TC01</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC01</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="13" t="inlineStr">
         <is>
           <t>The organiser sees how many places are taken and how many attendees have withdrawn</t>
         </is>
       </c>
-      <c r="D4" s="11" t="inlineStr">
+      <c r="D4" s="13" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="E4" s="11" t="inlineStr">
+      <c r="E4" s="13" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="10" t="inlineStr">
+    <row r="5" ht="25" customHeight="1">
+      <c r="A5" s="8" t="inlineStr">
         <is>
           <t>TC02</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC02</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="13" t="inlineStr">
         <is>
           <t>A registered attendee withdraws from My Registrations, and the registration is shown as Withdrawn</t>
         </is>
       </c>
-      <c r="D5" s="11" t="inlineStr">
+      <c r="D5" s="13" t="inlineStr">
         <is>
           <t>AC1, AC2</t>
         </is>
       </c>
-      <c r="E5" s="11" t="inlineStr">
+      <c r="E5" s="13" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="10" t="inlineStr">
+    <row r="6" ht="25" customHeight="1">
+      <c r="A6" s="8" t="inlineStr">
         <is>
           <t>TC03</t>
         </is>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC03</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C6" s="13" t="inlineStr">
         <is>
           <t>After withdrawing, the event page no longer shows the attendee as registered and offers Register instead</t>
         </is>
       </c>
-      <c r="D6" s="11" t="inlineStr">
+      <c r="D6" s="13" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="E6" s="11" t="inlineStr">
+      <c r="E6" s="13" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F6" s="11" t="inlineStr">
+      <c r="F6" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="A7" s="10" t="inlineStr">
+    <row r="7" ht="25" customHeight="1">
+      <c r="A7" s="8" t="inlineStr">
         <is>
           <t>TC04</t>
         </is>
       </c>
-      <c r="B7" s="11" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC04</t>
         </is>
       </c>
-      <c r="C7" s="11" t="inlineStr">
+      <c r="C7" s="13" t="inlineStr">
         <is>
           <t>The organiser and the coordinator see one place freed and one more withdrawal after an attendee withdraws</t>
         </is>
       </c>
-      <c r="D7" s="11" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>AC4, AC5</t>
         </is>
       </c>
-      <c r="E7" s="11" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F7" s="11" t="inlineStr">
+      <c r="F7" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="10" t="inlineStr">
+    <row r="8" ht="25" customHeight="1">
+      <c r="A8" s="8" t="inlineStr">
         <is>
           <t>TC05</t>
         </is>
       </c>
-      <c r="B8" s="11" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC05</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C8" s="13" t="inlineStr">
         <is>
           <t>Withdrawing from a full event from its event page frees the place, so another attendee can register</t>
         </is>
       </c>
-      <c r="D8" s="11" t="inlineStr">
+      <c r="D8" s="13" t="inlineStr">
         <is>
           <t>AC1, AC3, AC4</t>
         </is>
       </c>
-      <c r="E8" s="11" t="inlineStr">
+      <c r="E8" s="13" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F8" s="11" t="inlineStr">
+      <c r="F8" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="10" t="inlineStr">
+    <row r="9" ht="25" customHeight="1">
+      <c r="A9" s="8" t="inlineStr">
         <is>
           <t>TC06</t>
         </is>
       </c>
-      <c r="B9" s="11" t="inlineStr">
+      <c r="B9" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC06</t>
         </is>
       </c>
-      <c r="C9" s="11" t="inlineStr">
+      <c r="C9" s="13" t="inlineStr">
         <is>
           <t>Choosing 'Keep my place' in the withdraw dialog leaves the registration unchanged</t>
         </is>
       </c>
-      <c r="D9" s="11" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E9" s="11" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F9" s="11" t="inlineStr">
+      <c r="F9" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="10" t="inlineStr">
+    <row r="10" ht="25" customHeight="1">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>TC07</t>
         </is>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC07</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C10" s="13" t="inlineStr">
         <is>
           <t>Only a Registered registration offers Withdraw: waiting list, withdrawn and attended ones do not</t>
         </is>
       </c>
-      <c r="D10" s="11" t="inlineStr">
+      <c r="D10" s="13" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="E10" s="11" t="inlineStr">
+      <c r="E10" s="13" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F10" s="11" t="inlineStr">
+      <c r="F10" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="10" t="inlineStr">
+    <row r="11" ht="25" customHeight="1">
+      <c r="A11" s="8" t="inlineStr">
         <is>
           <t>TC08</t>
         </is>
       </c>
-      <c r="B11" s="11" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC08</t>
         </is>
       </c>
-      <c r="C11" s="11" t="inlineStr">
+      <c r="C11" s="13" t="inlineStr">
         <is>
           <t>After withdrawing from an event whose registration was turned off, the attendee can no longer open it</t>
         </is>
       </c>
-      <c r="D11" s="11" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>AC2, AC3</t>
         </is>
       </c>
-      <c r="E11" s="11" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Positive</t>
         </is>
       </c>
-      <c r="F11" s="11" t="inlineStr">
+      <c r="F11" s="13" t="inlineStr">
         <is>
           <t>Acceptance Criteria</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
+    <row r="12" ht="25" customHeight="1">
+      <c r="A12" s="8" t="inlineStr">
         <is>
           <t>TC09</t>
         </is>
       </c>
-      <c r="B12" s="11" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC09</t>
         </is>
       </c>
-      <c r="C12" s="11" t="inlineStr">
+      <c r="C12" s="13" t="inlineStr">
         <is>
           <t>The Ops Manager does not see the places taken or the withdrawals on the Registration card</t>
         </is>
       </c>
-      <c r="D12" s="11" t="inlineStr">
+      <c r="D12" s="13" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="E12" s="11" t="inlineStr">
+      <c r="E12" s="13" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F12" s="11" t="inlineStr">
+      <c r="F12" s="13" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="13" ht="25" customHeight="1">
+      <c r="A13" s="8" t="inlineStr">
         <is>
           <t>TC10</t>
         </is>
       </c>
-      <c r="B13" s="11" t="inlineStr">
+      <c r="B13" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC10</t>
         </is>
       </c>
-      <c r="C13" s="11" t="inlineStr">
+      <c r="C13" s="13" t="inlineStr">
         <is>
           <t>Withdrawing a second time from another open tab is refused, and the registration stays Withdrawn</t>
         </is>
       </c>
-      <c r="D13" s="11" t="inlineStr">
+      <c r="D13" s="13" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="E13" s="11" t="inlineStr">
+      <c r="E13" s="13" t="inlineStr">
         <is>
           <t>Negative</t>
         </is>
       </c>
-      <c r="F13" s="11" t="inlineStr">
+      <c r="F13" s="13" t="inlineStr">
         <is>
           <t>Code</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="10" t="inlineStr">
-        <is>
-          <t>TC11</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>SPM-52-TC11</t>
-        </is>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>Withdrawing on the event page of an event whose registration was turned off warns first, then shows the withdrawal on My Registrations instead of an error</t>
-        </is>
-      </c>
-      <c r="D14" s="11" t="inlineStr">
-        <is>
-          <t>AC1, AC2</t>
-        </is>
-      </c>
-      <c r="E14" s="11" t="inlineStr">
-        <is>
-          <t>Positive</t>
-        </is>
-      </c>
-      <c r="F14" s="11" t="inlineStr">
-        <is>
-          <t>Code</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="7" t="inlineStr">
+    <row r="16" ht="13" customHeight="1">
+      <c r="A16" s="16" t="inlineStr">
         <is>
           <t>AC</t>
         </is>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B16" s="16" t="inlineStr">
         <is>
           <t>Acceptance Criterion</t>
         </is>
       </c>
-      <c r="C17" s="8" t="n"/>
-      <c r="D17" s="9" t="n"/>
-      <c r="E17" s="7" t="inlineStr">
+      <c r="C16" s="14" t="n"/>
+      <c r="D16" s="15" t="n"/>
+      <c r="E16" s="16" t="inlineStr">
         <is>
           <t>Covered by</t>
         </is>
       </c>
-      <c r="F17" s="9" t="n"/>
-    </row>
-    <row r="18" ht="71.5" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="F16" s="15" t="n"/>
+    </row>
+    <row r="17" ht="58" customHeight="1">
+      <c r="A17" s="13" t="inlineStr">
         <is>
           <t>AC1</t>
         </is>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>A registered attendee can withdraw their registration.</t>
         </is>
       </c>
-      <c r="C18" s="8" t="n"/>
-      <c r="D18" s="9" t="n"/>
-      <c r="E18" s="11" t="inlineStr">
+      <c r="C17" s="14" t="n"/>
+      <c r="D17" s="15" t="n"/>
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC02
 SPM-52-TC05
 SPM-52-TC06
-SPM-52-TC07
-SPM-52-TC11</t>
-        </is>
-      </c>
-      <c r="F18" s="9" t="n"/>
-    </row>
-    <row r="19" ht="58" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
+SPM-52-TC07</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="n"/>
+    </row>
+    <row r="18" ht="44.5" customHeight="1">
+      <c r="A18" s="13" t="inlineStr">
         <is>
           <t>AC2</t>
         </is>
       </c>
-      <c r="B19" s="11" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>The registration status changes appropriately.</t>
         </is>
       </c>
-      <c r="C19" s="8" t="n"/>
-      <c r="D19" s="9" t="n"/>
-      <c r="E19" s="11" t="inlineStr">
+      <c r="C18" s="14" t="n"/>
+      <c r="D18" s="15" t="n"/>
+      <c r="E18" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC02
 SPM-52-TC08
-SPM-52-TC10
-SPM-52-TC11</t>
-        </is>
-      </c>
-      <c r="F19" s="9" t="n"/>
-    </row>
-    <row r="20" ht="44.5" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
+SPM-52-TC10</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="n"/>
+    </row>
+    <row r="19" ht="44.5" customHeight="1">
+      <c r="A19" s="13" t="inlineStr">
         <is>
           <t>AC3</t>
         </is>
       </c>
-      <c r="B20" s="11" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>The attendee can no longer be treated as an active registrant.</t>
         </is>
       </c>
-      <c r="C20" s="8" t="n"/>
-      <c r="D20" s="9" t="n"/>
-      <c r="E20" s="11" t="inlineStr">
+      <c r="C19" s="14" t="n"/>
+      <c r="D19" s="15" t="n"/>
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC03
 SPM-52-TC05
 SPM-52-TC08</t>
         </is>
       </c>
-      <c r="F20" s="9" t="n"/>
-    </row>
-    <row r="21" ht="31" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="F19" s="15" t="n"/>
+    </row>
+    <row r="20" ht="31" customHeight="1">
+      <c r="A20" s="13" t="inlineStr">
         <is>
           <t>AC4</t>
         </is>
       </c>
-      <c r="B21" s="11" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>The event's available capacity is updated where applicable.</t>
         </is>
       </c>
-      <c r="C21" s="8" t="n"/>
-      <c r="D21" s="9" t="n"/>
-      <c r="E21" s="11" t="inlineStr">
+      <c r="C20" s="14" t="n"/>
+      <c r="D20" s="15" t="n"/>
+      <c r="E20" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC04
 SPM-52-TC05</t>
         </is>
       </c>
-      <c r="F21" s="9" t="n"/>
-    </row>
-    <row r="22" ht="44.5" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
+      <c r="F20" s="15" t="n"/>
+    </row>
+    <row r="21" ht="44.5" customHeight="1">
+      <c r="A21" s="13" t="inlineStr">
         <is>
           <t>AC5</t>
         </is>
       </c>
-      <c r="B22" s="11" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Relevant Event Organisers or Coordinators can see the updated registration information.</t>
         </is>
       </c>
-      <c r="C22" s="8" t="n"/>
-      <c r="D22" s="9" t="n"/>
-      <c r="E22" s="11" t="inlineStr">
+      <c r="C21" s="14" t="n"/>
+      <c r="D21" s="15" t="n"/>
+      <c r="E21" s="13" t="inlineStr">
         <is>
           <t>SPM-52-TC01
 SPM-52-TC04
 SPM-52-TC09</t>
         </is>
       </c>
-      <c r="F22" s="9" t="n"/>
-    </row>
-    <row r="24" ht="179.5" customHeight="1">
-      <c r="A24" s="7" t="inlineStr">
+      <c r="F21" s="15" t="n"/>
+    </row>
+    <row r="23" ht="179.5" customHeight="1">
+      <c r="A23" s="16" t="inlineStr">
         <is>
           <t>Code reviewed</t>
         </is>
       </c>
-      <c r="B24" s="11" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>src/app/api/registrations/[id]/route.ts
 src/lib/registrationEligibility.ts
@@ -1026,40 +1025,39 @@
 scripts/seed-spm52.ts</t>
         </is>
       </c>
-      <c r="C24" s="8" t="n"/>
-      <c r="D24" s="8" t="n"/>
-      <c r="E24" s="8" t="n"/>
-      <c r="F24" s="9" t="n"/>
+      <c r="C23" s="14" t="n"/>
+      <c r="D23" s="14" t="n"/>
+      <c r="E23" s="14" t="n"/>
+      <c r="F23" s="15" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="14">
     <mergeCell ref="B19:D19"/>
     <mergeCell ref="E20:F20"/>
-    <mergeCell ref="E21:F21"/>
-    <mergeCell ref="B24:F24"/>
-    <mergeCell ref="B22:D22"/>
+    <mergeCell ref="E16:F16"/>
+    <mergeCell ref="B20:D20"/>
     <mergeCell ref="E19:F19"/>
     <mergeCell ref="B17:D17"/>
     <mergeCell ref="B18:D18"/>
-    <mergeCell ref="E22:F22"/>
+    <mergeCell ref="B23:F23"/>
     <mergeCell ref="B21:D21"/>
     <mergeCell ref="B1:F1"/>
     <mergeCell ref="E17:F17"/>
     <mergeCell ref="E18:F18"/>
-    <mergeCell ref="B20:D20"/>
+    <mergeCell ref="B16:D16"/>
+    <mergeCell ref="E21:F21"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A4" r:id="rId1"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A5" r:id="rId2"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A6" r:id="rId3"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A7" r:id="rId4"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A8" r:id="rId5"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A9" r:id="rId6"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A10" r:id="rId7"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A11" r:id="rId8"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A12" r:id="rId9"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A13" r:id="rId10"/>
-    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="A14" r:id="rId11"/>
+    <hyperlink ref="A4" location="'TC01'!A1" display="TC01"/>
+    <hyperlink ref="A5" location="'TC02'!A1" display="TC02"/>
+    <hyperlink ref="A6" location="'TC03'!A1" display="TC03"/>
+    <hyperlink ref="A7" location="'TC04'!A1" display="TC04"/>
+    <hyperlink ref="A8" location="'TC05'!A1" display="TC05"/>
+    <hyperlink ref="A9" location="'TC06'!A1" display="TC06"/>
+    <hyperlink ref="A10" location="'TC07'!A1" display="TC07"/>
+    <hyperlink ref="A11" location="'TC08'!A1" display="TC08"/>
+    <hyperlink ref="A12" location="'TC09'!A1" display="TC09"/>
+    <hyperlink ref="A13" location="'TC10'!A1" display="TC10"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1072,13 +1070,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1087,36 +1085,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC09</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>The Ops Manager does not see the places taken or the withdrawals on the Registration card</t>
         </is>
       </c>
     </row>
     <row r="4" ht="98.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm52` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM52 …' events, never anyone else's data).
 Logged in as Grace Lim (grace.lim@connectsphere.com / password123), the Ops Manager.
@@ -1125,12 +1123,12 @@
       </c>
     </row>
     <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'All Events' in the sidebar
 2. Click 'SPM52 Riverside Forum' in the list</t>
@@ -1138,53 +1136,52 @@
       </c>
     </row>
     <row r="6" ht="17.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Event: SPM52 Riverside Forum | Ops Manager: Grace Lim</t>
         </is>
       </c>
     </row>
     <row r="7" ht="44.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page opens. The Registration card shows 'Registration' Enabled, 'Capacity' 10, 'Opens' and 'Closes', but no 'Places taken' or 'Withdrawn' rows.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1193,19 +1190,19 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="37.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page opens. The Registration card shows 'Registration' Enabled, 'Capacity' 10, 'Opens' and 'Closes', but no 'Places taken' or 'Withdrawn' rows.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -1217,7 +1214,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -1229,7 +1226,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -1241,13 +1238,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -1263,13 +1260,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1278,36 +1275,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC10</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Withdrawing a second time from another open tab is refused, and the registration stays Withdrawn</t>
         </is>
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Before and after: run `npm run fixtures:spm52` (never `npx prisma db seed`, which wipes everyone's data).
 Logged in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee.</t>
@@ -1315,12 +1312,12 @@
       </c>
     </row>
     <row r="5" ht="166" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Open a new browser tab, type /registrations after the site address in its address bar (e.g. http://localhost:3000/registrations) and press Enter
@@ -1334,24 +1331,24 @@
       </c>
     </row>
     <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Attendee: Marcus Yeo | Event: SPM52 Riverside Forum | Two tabs of My Registrations</t>
         </is>
       </c>
     </row>
     <row r="7" ht="139" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 4: In the new tab, a green message says 'You have withdrawn from SPM52 Riverside Forum.' and the row's badge is 'Withdrawn'.
 Step 5: The first tab, not yet refreshed, still shows 'Registered'. A dialog asks 'Withdraw from SPM52 Riverside Forum?'.
@@ -1361,29 +1358,28 @@
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1392,13 +1388,13 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="100" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 4: In the new tab, a green message says 'You have withdrawn from SPM52 Riverside Forum.' and the row's badge is 'Withdrawn'.
 Step 5: The first tab, not yet refreshed, still shows 'Registered'. A dialog asks 'Withdraw from SPM52 Riverside Forum?'.
@@ -1407,7 +1403,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -1419,7 +1415,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -1431,7 +1427,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -1443,13 +1439,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -1465,13 +1461,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1480,107 +1476,110 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
-        <is>
-          <t>SPM-52-TC11</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="44.5" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
+        <is>
+          <t>SPM-52-BUG-TC01</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="31" customHeight="1">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Withdrawing on the event page of an event whose registration was turned off warns first, then shows the withdrawal on My Registrations instead of an error</t>
+      <c r="B3" s="11" t="inlineStr">
+        <is>
+          <t>After withdrawing from an event whose registration was turned off, the attendee can no longer open it</t>
         </is>
       </c>
     </row>
     <row r="4" ht="71.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Before and after: run `npm run fixtures:spm52` (never `npx prisma db seed`, which wipes everyone's data).
 Logged in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee. 'SPM52 Members Gala' had its registration turned off after he registered.</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+    <row r="5" ht="85" customHeight="1">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Click the 'SPM52 Members Gala' row
-3. Click 'Withdraw' in the 'Your registration' card
-4. Click 'Withdraw' in the dialog</t>
+3. Click 'My Registrations' in the sidebar
+4. Click 'Withdraw' on the 'SPM52 Members Gala' row
+5. Click 'Withdraw' in the dialog
+6. Click the 'SPM52 Members Gala' row</t>
         </is>
       </c>
     </row>
     <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Attendee: Marcus Yeo | Event: SPM52 Members Gala (registration not enabled)</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="166" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="7" ht="230" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Step 2: The event page opens. The Registration card says 'Not enabled for this event'; the 'Your registration' card shows the badge 'Registered' and a 'Withdraw' button.
-Step 3: A dialog asks 'Withdraw from SPM52 Members Gala?' and warns, in yellow, 'Registration for this event has been turned off, so you can't register again. Once you withdraw, you won't be able to open this event any more.', with the buttons 'Keep my place' and 'Withdraw'.
-Step 4: The 'My Registrations' page opens. A green message says 'You have withdrawn from SPM52 Members Gala.' and the row's badge is 'Withdrawn'. No 'This event doesn't exist, or you don't have access to it.' message is shown.</t>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Step 1: 'SPM52 Members Gala' is listed with the badge 'Registered' and a 'Withdraw' button.
+Step 2: The event page opens. The Registration card says 'Not enabled for this event'; the 'Your registration' card shows the badge 'Registered' and a 'Withdraw' button.
+Step 4: A dialog asks 'Withdraw from SPM52 Members Gala?' and warns, in yellow, 'Registration for this event has been turned off, so you can't register again. Once you withdraw, you won't be able to open this event any more.'
+Step 5: A green message says 'You have withdrawn from SPM52 Members Gala.' and the row's badge is now 'Withdrawn'.
+Step 6: The page says 'This event doesn't exist, or you don't have access to it.' - he no longer holds a place, so the event is no longer shown to him.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
-        <v>46310</v>
-      </c>
-    </row>
-    <row r="10"/>
-    <row r="11">
+      <c r="B9" s="12" t="n">
+        <v>46311</v>
+      </c>
+    </row>
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1589,45 +1588,67 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="230" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Step 1: 'SPM52 Members Gala' is listed with the badge 'Registered' and a 'Withdraw' button.
+Step 2: The event page opens. The Registration card says 'Not enabled for this event'; the 'Your registration' card shows the badge 'Registered' and a 'Withdraw' button.
+Step 4: A dialog asks 'Withdraw from SPM52 Members Gala?' and warns, in yellow, 'Registration for this event has been turned off, so you can't register again. Once you withdraw, you won't be able to open this event any more.'
+Step 5: A green message says 'You have withdrawn from SPM52 Members Gala.' and the row's badge is now 'Withdrawn'.
+Step 6: The page says 'This event doesn't exist, or you don't have access to it.' - he no longer holds a place, so the event is no longer shown to him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-    <row r="16">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="12" t="n">
+        <v>46311</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1641,13 +1662,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1656,36 +1677,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC01</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>The organiser sees how many places are taken and how many attendees have withdrawn</t>
         </is>
       </c>
     </row>
     <row r="4" ht="112" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm52` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM52 …' events, never anyone else's data), and nobody has withdrawn from 'SPM52 Riverside Forum' since.
 Logged in as Evelyn Chen (evelyn.chen@straitsmedic.com / password123), who organised every 'SPM52 …' event.
@@ -1694,12 +1715,12 @@
       </c>
     </row>
     <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Events' in the sidebar
 2. Click 'SPM52 Riverside Forum' in the list</t>
@@ -1707,53 +1728,52 @@
       </c>
     </row>
     <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Event: SPM52 Riverside Forum (capacity 10; 4 registered, 1 withdrawn) | Organiser: Evelyn Chen</t>
         </is>
       </c>
     </row>
     <row r="7" ht="58" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page opens with the heading 'SPM52 Riverside Forum'. The Registration card shows 'Registration' Enabled, 'Capacity' 10, 'Places taken' '4 of 10 · 6 left' and 'Withdrawn' '1'.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1762,19 +1782,19 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="37.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page opens with the heading 'SPM52 Riverside Forum'. The Registration card shows 'Registration' Enabled, 'Capacity' 10, 'Places taken' '4 of 10 · 6 left' and 'Withdrawn' '1'.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -1786,7 +1806,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -1798,7 +1818,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -1810,13 +1830,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -1832,13 +1852,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1847,36 +1867,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC02</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>A registered attendee withdraws from My Registrations, and the registration is shown as Withdrawn</t>
         </is>
       </c>
     </row>
     <row r="4" ht="85" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Before: run `npm run fixtures:spm52` (never `npx prisma db seed`, which wipes everyone's data).
 Do not reset after: SPM-52-TC03 and SPM-52-TC04 continue from this withdrawal; reset after SPM-52-TC04.
@@ -1885,12 +1905,12 @@
       </c>
     </row>
     <row r="5" ht="58" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Click 'Withdraw' on the 'SPM52 Riverside Forum' row
@@ -1900,24 +1920,24 @@
       </c>
     </row>
     <row r="6" ht="17.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Attendee: Marcus Yeo | Event: SPM52 Riverside Forum</t>
         </is>
       </c>
     </row>
     <row r="7" ht="179.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 1: The 'My Registrations' page lists 'SPM52 Riverside Forum' (4 Mar 2028, 09:00–17:00) with the badge 'Registered' and a 'Withdraw' button.
 Step 2: The event page does not open. A dialog asks 'Withdraw from SPM52 Riverside Forum?' and says 'Your place is released and can be taken by someone else. To attend, you would have to register again, and the event may be full by then.', with the buttons 'Keep my place' and 'Withdraw'.
@@ -1927,29 +1947,28 @@
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -1958,13 +1977,13 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="162.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 1: The 'My Registrations' page lists 'SPM52 Riverside Forum' (4 Mar 2028, 09:00–17:00) with the badge 'Registered' and a 'Withdraw' button.
 Step 2: The event page does not open. A dialog asks 'Withdraw from SPM52 Riverside Forum?' and says 'Your place is released and can be taken by someone else. To attend, you would have to register again, and the event may be full by then.', with the buttons 'Keep my place' and 'Withdraw'.
@@ -1973,7 +1992,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -1985,7 +2004,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -1997,7 +2016,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -2009,13 +2028,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -2031,13 +2050,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2046,36 +2065,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC03</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>After withdrawing, the event page no longer shows the attendee as registered and offers Register instead</t>
         </is>
       </c>
     </row>
     <row r="4" ht="98.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC02 has just been run (Marcus Yeo has withdrawn from 'SPM52 Riverside Forum').
 Do not reset after: SPM-52-TC04 continues from the same withdrawal.
@@ -2085,12 +2104,12 @@
       </c>
     </row>
     <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Click the 'SPM52 Riverside Forum' row</t>
@@ -2098,53 +2117,52 @@
       </c>
     </row>
     <row r="6" ht="17.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Attendee: Marcus Yeo | Event: SPM52 Riverside Forum</t>
         </is>
       </c>
     </row>
     <row r="7" ht="71.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page 'SPM52 Riverside Forum' opens. The 'Your registration' card shows the 'Dietary requirements' and 'Accessibility requirements' fields and a 'Register' button. It shows no 'Registered' badge, no 'You registered on …' line and no 'Withdraw' button.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2153,19 +2171,19 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="50" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page 'SPM52 Riverside Forum' opens. The 'Your registration' card shows the 'Dietary requirements' and 'Accessibility requirements' fields and a 'Register' button. It shows no 'Registered' badge, no 'You registered on …' line and no 'Withdraw' button.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -2177,7 +2195,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -2189,7 +2207,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -2201,13 +2219,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -2223,13 +2241,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2238,36 +2256,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC04</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>The organiser and the coordinator see one place freed and one more withdrawal after an attendee withdraws</t>
         </is>
       </c>
     </row>
     <row r="4" ht="71.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC03 has just been run (it follows SPM-52-TC02, in which Marcus Yeo withdrew from 'SPM52 Riverside Forum').
 After: run `npm run fixtures:spm52` (never `npx prisma db seed`, which wipes everyone's data).
@@ -2276,12 +2294,12 @@
       </c>
     </row>
     <row r="5" ht="125.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Log out and log in as Evelyn Chen (evelyn.chen@straitsmedic.com / password123), who organised every 'SPM52 …' event
 2. Click 'My Events' in the sidebar
@@ -2293,24 +2311,24 @@
       </c>
     </row>
     <row r="6" ht="44.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Event: SPM52 Riverside Forum (capacity 10; now 3 registered, 2 withdrawn) | Organiser: Evelyn Chen | Coordinator: Daniel Tan</t>
         </is>
       </c>
     </row>
     <row r="7" ht="71.5" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 3: The Registration card shows 'Places taken' '3 of 10 · 7 left' and 'Withdrawn' '2' (it was '4 of 10 · 6 left' and '1' before Marcus Yeo withdrew).
 Step 6: The Registration card shows 'Places taken' '3 of 10 · 7 left' and 'Withdrawn' '2'.</t>
@@ -2318,29 +2336,28 @@
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2349,20 +2366,20 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="62.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 3: The Registration card shows 'Places taken' '3 of 10 · 7 left' and 'Withdrawn' '2' (it was '4 of 10 · 6 left' and '1' before Marcus Yeo withdrew).
 Step 6: The Registration card shows 'Places taken' '3 of 10 · 7 left' and 'Withdrawn' '2'.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -2374,7 +2391,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -2386,7 +2403,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -2398,13 +2415,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -2420,13 +2437,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2435,36 +2452,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC05</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Withdrawing from a full event from its event page frees the place, so another attendee can register</t>
         </is>
       </c>
     </row>
     <row r="4" ht="58" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Before and after: run `npm run fixtures:spm52` (never `npx prisma db seed`, which wipes everyone's data).
 Logged in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee.</t>
@@ -2472,12 +2489,12 @@
       </c>
     </row>
     <row r="5" ht="139" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'Browse Events' in the sidebar
 2. Click 'SPM52 Last Place Clinic'
@@ -2492,24 +2509,24 @@
       </c>
     </row>
     <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Event: SPM52 Last Place Clinic (capacity 2; Marcus Yeo and Anita Devi registered) | Attendees: Marcus Yeo, Tan Jia Hui</t>
         </is>
       </c>
     </row>
     <row r="7" ht="220" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 1: 'SPM52 Last Place Clinic' is listed with the badge 'Full'.
 Step 2: The event page opens. The 'Your registration' card shows the badge 'Registered', 'You registered on &lt;date&gt;.' and a 'Withdraw' button.
@@ -2522,29 +2539,28 @@
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2553,13 +2569,13 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="175" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 1: 'SPM52 Last Place Clinic' is listed with the badge 'Full'.
 Step 2: The event page opens. The 'Your registration' card shows the badge 'Registered', 'You registered on &lt;date&gt;.' and a 'Withdraw' button.
@@ -2571,7 +2587,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -2583,7 +2599,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -2595,7 +2611,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -2607,13 +2623,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -2629,13 +2645,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2644,36 +2660,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC06</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Choosing 'Keep my place' in the withdraw dialog leaves the registration unchanged</t>
         </is>
       </c>
     </row>
     <row r="4" ht="98.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm52` has been run from the project folder since the last full `npx prisma db seed`, and since SPM-52-TC02 was last run (Marcus Yeo holds his place on 'SPM52 Riverside Forum').
 Logged in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee.
@@ -2682,12 +2698,12 @@
       </c>
     </row>
     <row r="5" ht="71.5" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Click the 'SPM52 Riverside Forum' row
@@ -2698,24 +2714,24 @@
       </c>
     </row>
     <row r="6" ht="17.5" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Attendee: Marcus Yeo | Event: SPM52 Riverside Forum</t>
         </is>
       </c>
     </row>
     <row r="7" ht="166" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page opens. The 'Your registration' card shows the badge 'Registered', 'You registered on &lt;date&gt;.' and a 'Withdraw' button. The Registration card has no 'Places taken' or 'Withdrawn' rows (they are for the organiser and coordinator).
 Step 3: A dialog asks 'Withdraw from SPM52 Riverside Forum?'.
@@ -2725,29 +2741,28 @@
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2756,13 +2771,13 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="125" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 2: The event page opens. The 'Your registration' card shows the badge 'Registered', 'You registered on &lt;date&gt;.' and a 'Withdraw' button. The Registration card has no 'Places taken' or 'Withdrawn' rows (they are for the organiser and coordinator).
 Step 3: A dialog asks 'Withdraw from SPM52 Riverside Forum?'.
@@ -2771,7 +2786,7 @@
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -2783,7 +2798,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -2795,7 +2810,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -2807,13 +2822,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -2829,13 +2844,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2844,36 +2859,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC07</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>Only a Registered registration offers Withdraw: waiting list, withdrawn and attended ones do not</t>
         </is>
       </c>
     </row>
     <row r="4" ht="98.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Test data loaded: `npm run fixtures:spm52` has been run from the project folder since the last full `npx prisma db seed` (it only touches the 'SPM52 …' events, never anyone else's data).
 Logged in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee.
@@ -2882,12 +2897,12 @@
       </c>
     </row>
     <row r="5" ht="31" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Click the 'SPM52 Waiting List Workshop' row</t>
@@ -2895,24 +2910,24 @@
       </c>
     </row>
     <row r="6" ht="58" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Attendee: Marcus Yeo | Events: SPM52 Waiting List Workshop (waiting list), SPM52 Dropped Plans Seminar (withdrawn), SPM52 Past Wellness Clinic (attended), SPM52 Riverside Forum (registered)</t>
         </is>
       </c>
     </row>
     <row r="7" ht="112" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 1: 'SPM52 Waiting List Workshop' has the badge 'Waiting list', 'SPM52 Dropped Plans Seminar' has 'Withdrawn' and 'SPM52 Past Wellness Clinic' has 'Attended'; none of the three has a 'Withdraw' button. 'SPM52 Riverside Forum' ('Registered') does.
 Step 2: The event page opens. The 'Your registration' card shows the badge 'Waiting list' and 'You're on the waiting list.', with no 'Withdraw' button.</t>
@@ -2920,29 +2935,28 @@
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -2951,20 +2965,20 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="87.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="inlineStr">
+      <c r="B12" s="11" t="inlineStr">
         <is>
           <t>Step 1: 'SPM52 Waiting List Workshop' has the badge 'Waiting list', 'SPM52 Dropped Plans Seminar' has 'Withdrawn' and 'SPM52 Past Wellness Clinic' has 'Attended'; none of the three has a 'Withdraw' button. 'SPM52 Riverside Forum' ('Registered') does.
 Step 2: The event page opens. The 'Your registration' card shows the badge 'Waiting list' and 'You're on the waiting list.', with no 'Withdraw' button.</t>
         </is>
       </c>
     </row>
-    <row r="13">
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
@@ -2976,7 +2990,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
@@ -2988,7 +3002,7 @@
         </is>
       </c>
     </row>
-    <row r="15">
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
@@ -3000,13 +3014,13 @@
         </is>
       </c>
     </row>
-    <row r="16">
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="15" t="n">
+      <c r="B16" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
@@ -3022,13 +3036,13 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:C16"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
-    <col width="24.77734375" customWidth="1" min="1" max="1"/>
-    <col width="56.77734375" customWidth="1" min="2" max="2"/>
+    <col width="24.81640625" customWidth="1" min="1" max="1"/>
+    <col width="56.81640625" customWidth="1" min="2" max="2"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="13" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
@@ -3037,36 +3051,36 @@
       <c r="B1" s="2" t="n"/>
     </row>
     <row r="2" ht="17.5" customHeight="1">
-      <c r="A2" s="12" t="inlineStr">
+      <c r="A2" s="10" t="inlineStr">
         <is>
           <t>Test Case ID</t>
         </is>
       </c>
-      <c r="B2" s="13" t="inlineStr">
+      <c r="B2" s="11" t="inlineStr">
         <is>
           <t>SPM-52-TC08</t>
         </is>
       </c>
     </row>
     <row r="3" ht="31" customHeight="1">
-      <c r="A3" s="12" t="inlineStr">
+      <c r="A3" s="10" t="inlineStr">
         <is>
           <t>Summary</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
+      <c r="B3" s="11" t="inlineStr">
         <is>
           <t>After withdrawing from an event whose registration was turned off, the attendee can no longer open it</t>
         </is>
       </c>
     </row>
     <row r="4" ht="71.5" customHeight="1">
-      <c r="A4" s="12" t="inlineStr">
+      <c r="A4" s="10" t="inlineStr">
         <is>
           <t>Pre-conditions</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
+      <c r="B4" s="11" t="inlineStr">
         <is>
           <t>Before and after: run `npm run fixtures:spm52` (never `npx prisma db seed`, which wipes everyone's data).
 Logged in as Marcus Yeo (marcus.yeo@example.com / password123), an Attendee. 'SPM52 Members Gala' had its registration turned off after he registered.</t>
@@ -3074,12 +3088,12 @@
       </c>
     </row>
     <row r="5" ht="85" customHeight="1">
-      <c r="A5" s="12" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>Test Steps</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>1. Click 'My Registrations' in the sidebar
 2. Click the 'SPM52 Members Gala' row
@@ -3091,57 +3105,56 @@
       </c>
     </row>
     <row r="6" ht="31" customHeight="1">
-      <c r="A6" s="12" t="inlineStr">
+      <c r="A6" s="10" t="inlineStr">
         <is>
           <t>Test Data</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="11" t="inlineStr">
         <is>
           <t>Attendee: Marcus Yeo | Event: SPM52 Members Gala (registration not enabled)</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="193" customHeight="1">
-      <c r="A7" s="12" t="inlineStr">
+    <row r="7" ht="152.5" customHeight="1">
+      <c r="A7" s="10" t="inlineStr">
         <is>
           <t>Expected Result</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Step 1: 'SPM52 Members Gala' is listed with the badge 'Registered' and a 'Withdraw' button.
 Step 2: The event page opens. The Registration card says 'Not enabled for this event'; the 'Your registration' card shows the badge 'Registered' and a 'Withdraw' button.
-Step 4: A dialog asks 'Withdraw from SPM52 Members Gala?' and warns, in yellow, 'Registration for this event has been turned off, so you can't register again. Once you withdraw, you won't be able to open this event any more.'
+Step 4: A dialog asks 'Withdraw from SPM52 Members Gala?'.
 Step 5: A green message says 'You have withdrawn from SPM52 Members Gala.' and the row's badge is now 'Withdrawn'.
 Step 6: The page says 'This event doesn't exist, or you don't have access to it.' - he no longer holds a place, so the event is no longer shown to him.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="17.5" customHeight="1">
-      <c r="A8" s="12" t="inlineStr">
+      <c r="A8" s="10" t="inlineStr">
         <is>
           <t>Created By</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="11" t="inlineStr">
         <is>
           <t>Sammi Chua</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="12" t="inlineStr">
+    <row r="9" ht="12.5" customHeight="1">
+      <c r="A9" s="10" t="inlineStr">
         <is>
           <t>Creation Date</t>
         </is>
       </c>
-      <c r="B9" s="14" t="n">
+      <c r="B9" s="12" t="n">
         <v>46310</v>
       </c>
     </row>
-    <row r="10"/>
-    <row r="11">
+    <row r="11" ht="13" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>Item</t>
@@ -3150,45 +3163,67 @@
       <c r="B11" s="5" t="n"/>
       <c r="C11" s="6" t="n"/>
     </row>
-    <row r="12">
+    <row r="12" ht="137.5" customHeight="1">
       <c r="A12" s="3" t="inlineStr">
         <is>
           <t>Actual Result</t>
         </is>
       </c>
-      <c r="B12" s="3" t="n"/>
-    </row>
-    <row r="13">
+      <c r="B12" s="11" t="inlineStr">
+        <is>
+          <t>Step 1: 'SPM52 Members Gala' is listed with the badge 'Registered' and a 'Withdraw' button.
+Step 2: The event page opens. The Registration card says 'Not enabled for this event'; the 'Your registration' card shows the badge 'Registered' and a 'Withdraw' button.
+Step 4: A dialog asks 'Withdraw from SPM52 Members Gala?'.
+Step 5: A green message says 'You have withdrawn from SPM52 Members Gala.' and the row's badge is now 'Withdrawn'.
+Step 6: The page says 'This event doesn't exist, or you don't have access to it.' - he no longer holds a place, so the event is no longer shown to him.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="12.5" customHeight="1">
       <c r="A13" s="3" t="inlineStr">
         <is>
           <t>Pass/Fail/Not Executed/Blocked</t>
         </is>
       </c>
-      <c r="B13" s="3" t="n"/>
-    </row>
-    <row r="14">
+      <c r="B13" s="3" t="inlineStr">
+        <is>
+          <t>Pass</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="12.5" customHeight="1">
       <c r="A14" s="3" t="inlineStr">
         <is>
           <t>Remarks</t>
         </is>
       </c>
-      <c r="B14" s="3" t="n"/>
-    </row>
-    <row r="15">
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>NA</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="12.5" customHeight="1">
       <c r="A15" s="3" t="inlineStr">
         <is>
           <t>Executed by</t>
         </is>
       </c>
-      <c r="B15" s="3" t="n"/>
-    </row>
-    <row r="16">
+      <c r="B15" s="3" t="inlineStr">
+        <is>
+          <t>Sammi</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="12.5" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
           <t>Date of Execution</t>
         </is>
       </c>
-      <c r="B16" s="3" t="n"/>
+      <c r="B16" s="12" t="n">
+        <v>46310</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>